<commit_message>
Fix tài liệu SOP tránh dịch thừa
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-161_ECR_ECO.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-161_ECR_ECO.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM161_ECRECO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM161_ImplPlan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM161_ImplPlan" sheetId="2" state="veryHidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM161_Evidence" sheetId="3" state="veryHidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zLISTS" sheetId="4" state="veryHidden" r:id="rId4"/>
   </sheets>
@@ -2750,8 +2750,8 @@
   </sheetData>
   <mergeCells count="70">
     <mergeCell ref="L4:AP4"/>
+    <mergeCell ref="K11:AB11"/>
     <mergeCell ref="AQ3:AV3"/>
-    <mergeCell ref="K11:AB11"/>
     <mergeCell ref="K20:AB20"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="AC9:AL9"/>

</xml_diff>